<commit_message>
fix(privacy): remove real customer and location data from the public repo
This repository is public. Three tracked files carried data from an actual
deployment area:

- scripts/generate_test_pdfs.cjs contained a real customer name ("Franz
  Mendl", also in two output filenames) and the real project cluster
  ("Herrieden"). The file is a standalone re-implementation of the protocol
  layout that drifts from the actual PdfExporter output, so it is untracked
  rather than sanitised, and generate_*_pdfs.cjs is now ignored.
- src/example-data/Beispiel-Kundenliste.xlsx and electron/CustomerStore.ts
  used the real postal codes of the deployment area (91567, 91572) in
  otherwise fictional demo records; replaced with 12345 / 12346.

Also ignore *.sor and *.pdf so measurement files and generated protocols
cannot be committed by accident.
</commit_message>
<xml_diff>
--- a/src/example-data/Beispiel-Kundenliste.xlsx
+++ b/src/example-data/Beispiel-Kundenliste.xlsx
@@ -43,16 +43,16 @@
     <t>Am Stadtpark 14</t>
   </si>
   <si>
-    <t>91567 Musterstadt</t>
+    <t>12345 Musterstadt</t>
   </si>
   <si>
     <t>NVt 01 (KVz-1) ➔ HÜP Mustermann (WE 01)</t>
   </si>
   <si>
-    <t>K-91567-NVT01-HUEP01</t>
-  </si>
-  <si>
-    <t>AUFTRAG-91567-10001</t>
+    <t>K-12345-NVT01-HUEP01</t>
+  </si>
+  <si>
+    <t>AUFTRAG-12345-10001</t>
   </si>
   <si>
     <t>Erika Beispiel</t>
@@ -64,10 +64,10 @@
     <t>NVt 01 (KVz-1) ➔ HÜP Beispiel (WE 02)</t>
   </si>
   <si>
-    <t>K-91567-NVT01-HUEP02</t>
-  </si>
-  <si>
-    <t>AUFTRAG-91567-10002</t>
+    <t>K-12345-NVT01-HUEP02</t>
+  </si>
+  <si>
+    <t>AUFTRAG-12345-10002</t>
   </si>
   <si>
     <t>Familie Musterhausen</t>
@@ -79,10 +79,10 @@
     <t>NVt 02 (KVz-1) ➔ HÜP Musterhausen (WE 03)</t>
   </si>
   <si>
-    <t>K-91567-NVT02-HUEP03</t>
-  </si>
-  <si>
-    <t>AUFTRAG-91567-10003</t>
+    <t>K-12345-NVT02-HUEP03</t>
+  </si>
+  <si>
+    <t>AUFTRAG-12345-10003</t>
   </si>
   <si>
     <t>Petra Testfrau</t>
@@ -91,16 +91,16 @@
     <t>Am Musterhof 5</t>
   </si>
   <si>
-    <t>91572 Beispieldorf</t>
+    <t>12346 Beispieldorf</t>
   </si>
   <si>
     <t>NVt 02 (KVz-1) ➔ HÜP Testfrau (WE 04)</t>
   </si>
   <si>
-    <t>K-91572-NVT02-HUEP04</t>
-  </si>
-  <si>
-    <t>AUFTRAG-91572-10004</t>
+    <t>K-12346-NVT02-HUEP04</t>
+  </si>
+  <si>
+    <t>AUFTRAG-12346-10004</t>
   </si>
   <si>
     <t>Thomas Vorlage</t>
@@ -112,10 +112,10 @@
     <t>NVt 03 (KVz-2) ➔ HÜP Vorlage (WE 05)</t>
   </si>
   <si>
-    <t>K-91572-NVT03-HUEP05</t>
-  </si>
-  <si>
-    <t>AUFTRAG-91572-10005</t>
+    <t>K-12346-NVT03-HUEP05</t>
+  </si>
+  <si>
+    <t>AUFTRAG-12346-10005</t>
   </si>
   <si>
     <t>Sabine Schablone</t>
@@ -127,10 +127,10 @@
     <t>NVt 03 (KVz-2) ➔ HÜP Schablone (WE 06)</t>
   </si>
   <si>
-    <t>K-91572-NVT03-HUEP06</t>
-  </si>
-  <si>
-    <t>AUFTRAG-91572-10006</t>
+    <t>K-12346-NVT03-HUEP06</t>
+  </si>
+  <si>
+    <t>AUFTRAG-12346-10006</t>
   </si>
 </sst>
 </file>
@@ -708,6 +708,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>